<commit_message>
Fix global-error.tsx: remove Sentry import to resolve Next.js CI build failure
</commit_message>
<xml_diff>
--- a/Rapport_Tests_E2E_Microservices.xlsx
+++ b/Rapport_Tests_E2E_Microservices.xlsx
@@ -1,12 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D564B1C-6BFB-4913-BFDA-0C3B3703443D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView minimized="1" xWindow="372" yWindow="372" windowWidth="23016" windowHeight="12216" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="📊 Résumé Global" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="🟢 Tests Jest (Unit &amp; Intégrati" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="🌐 Tests E2E Playwright" state="visible" r:id="rId6"/>
+    <sheet name="📊 Résumé Global" sheetId="1" r:id="rId1"/>
+    <sheet name="🟢 Tests Jest (Unit &amp; Intégrati" sheetId="2" r:id="rId2"/>
+    <sheet name="🌐 Tests E2E Playwright" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -489,45 +493,55 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="8" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF666666"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="13"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF666666"/>
-      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <b/>
       <color rgb="FF27AE60"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="8">
@@ -597,12 +611,6 @@
   </cellStyleXfs>
   <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -627,6 +635,12 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -965,27 +979,27 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="45" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="1" max="1" width="32.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="73.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:2" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-    </row>
-    <row r="2" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="17"/>
+    </row>
+    <row r="2" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B2" s="18"/>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -993,39 +1007,39 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:2" s="1" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -1033,40 +1047,40 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" ht="25" customHeight="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
+    <row r="9" spans="1:2" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B10" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B11" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B12" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B13" t="s">
@@ -1079,14 +1093,14 @@
     <mergeCell ref="A2:B2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F43"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -1096,876 +1110,876 @@
     <col min="6" max="6" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:6" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:6" s="4" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
+    <row r="2" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F2" s="9" t="s">
+      <c r="E2" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" s="7" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+    <row r="3" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F3" s="12" t="s">
+      <c r="E3" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="10" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+    <row r="4" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="E4" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F4" s="9" t="s">
+      <c r="E4" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+    <row r="5" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="E5" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5" s="12" t="s">
+      <c r="E5" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" s="10" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
+    <row r="6" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="E6" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6" s="9" t="s">
+      <c r="E6" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" s="7" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="7" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+    <row r="7" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="E7" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F7" s="12" t="s">
+      <c r="E7" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" s="10" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
+    <row r="8" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F8" s="9" t="s">
+      <c r="E8" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" s="7" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
+    <row r="9" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F9" s="12" t="s">
+      <c r="E9" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" s="10" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
+    <row r="10" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E10" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F10" s="9" t="s">
+      <c r="E10" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" s="7" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
+    <row r="11" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="E11" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F11" s="12" t="s">
+      <c r="E11" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F11" s="10" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
+    <row r="12" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E12" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F12" s="9" t="s">
+      <c r="E12" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F12" s="7" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="12" t="s">
+    <row r="13" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" s="12" t="s">
+      <c r="B13" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="E13" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F13" s="12" t="s">
+      <c r="E13" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F13" s="10" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
+    <row r="14" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C14" s="9" t="s">
+      <c r="B14" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F14" s="9" t="s">
+      <c r="E14" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F14" s="7" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
+    <row r="15" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C15" s="12" t="s">
+      <c r="B15" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D15" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="E15" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F15" s="12" t="s">
+      <c r="E15" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F15" s="10" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="9" t="s">
+    <row r="16" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C16" s="9" t="s">
+      <c r="B16" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="E16" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F16" s="9" t="s">
+      <c r="E16" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F16" s="7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
+    <row r="17" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C17" s="12" t="s">
+      <c r="B17" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D17" s="12" t="s">
+      <c r="D17" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="E17" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F17" s="12" t="s">
+      <c r="E17" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F17" s="10" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="18" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
+    <row r="18" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C18" s="9" t="s">
+      <c r="B18" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="D18" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="E18" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F18" s="9" t="s">
+      <c r="E18" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F18" s="7" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
+    <row r="19" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B19" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C19" s="12" t="s">
+      <c r="B19" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D19" s="12" t="s">
+      <c r="D19" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="E19" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F19" s="12" t="s">
+      <c r="E19" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F19" s="10" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="20" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="9" t="s">
+    <row r="20" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C20" s="9" t="s">
+      <c r="B20" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="D20" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="E20" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F20" s="9" t="s">
+      <c r="E20" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F20" s="7" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="21" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="12" t="s">
+    <row r="21" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B21" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C21" s="12" t="s">
+      <c r="B21" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="D21" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="E21" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F21" s="12" t="s">
+      <c r="E21" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F21" s="10" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="22" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="9" t="s">
+    <row r="22" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B22" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C22" s="9" t="s">
+      <c r="B22" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="D22" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="E22" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F22" s="9" t="s">
+      <c r="E22" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F22" s="7" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="23" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="12" t="s">
+    <row r="23" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C23" s="12" t="s">
+      <c r="B23" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D23" s="12" t="s">
+      <c r="D23" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="E23" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F23" s="12" t="s">
+      <c r="E23" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F23" s="10" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="9" t="s">
+    <row r="24" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B24" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C24" s="9" t="s">
+      <c r="B24" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C24" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="D24" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="E24" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F24" s="9" t="s">
+      <c r="E24" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F24" s="7" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="25" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="12" t="s">
+    <row r="25" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B25" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C25" s="12" t="s">
+      <c r="B25" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D25" s="12" t="s">
+      <c r="D25" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="E25" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F25" s="12" t="s">
+      <c r="E25" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F25" s="10" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="26" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="9" t="s">
+    <row r="26" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C26" s="9" t="s">
+      <c r="B26" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="E26" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F26" s="9" t="s">
+      <c r="E26" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F26" s="7" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="27" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="12" t="s">
+    <row r="27" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B27" s="12" t="s">
+      <c r="B27" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="C27" s="12" t="s">
+      <c r="C27" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="D27" s="12" t="s">
+      <c r="D27" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="E27" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F27" s="12" t="s">
+      <c r="E27" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F27" s="10" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="28" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="9" t="s">
+    <row r="28" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="B28" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C28" s="9" t="s">
+      <c r="C28" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="D28" s="9" t="s">
+      <c r="D28" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="E28" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F28" s="9" t="s">
+      <c r="E28" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F28" s="7" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="29" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="12" t="s">
+    <row r="29" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B29" s="12" t="s">
+      <c r="B29" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="12" t="s">
+      <c r="C29" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="D29" s="12" t="s">
+      <c r="D29" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E29" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F29" s="12" t="s">
+      <c r="E29" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F29" s="10" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="30" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="9" t="s">
+    <row r="30" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="D30" s="9" t="s">
+      <c r="D30" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="E30" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F30" s="9" t="s">
+      <c r="E30" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F30" s="7" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="31" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="12" t="s">
+    <row r="31" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B31" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C31" s="12" t="s">
+      <c r="B31" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C31" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="D31" s="12" t="s">
+      <c r="D31" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="E31" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F31" s="12" t="s">
+      <c r="E31" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F31" s="10" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="32" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="9" t="s">
+    <row r="32" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B32" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C32" s="9" t="s">
+      <c r="B32" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C32" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="D32" s="9" t="s">
+      <c r="D32" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="E32" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F32" s="9" t="s">
+      <c r="E32" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F32" s="7" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="33" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="12" t="s">
+    <row r="33" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B33" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C33" s="12" t="s">
+      <c r="B33" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C33" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="D33" s="12" t="s">
+      <c r="D33" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="E33" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F33" s="12" t="s">
+      <c r="E33" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F33" s="10" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="34" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="9" t="s">
+    <row r="34" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B34" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C34" s="9" t="s">
+      <c r="B34" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C34" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="D34" s="9" t="s">
+      <c r="D34" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="E34" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F34" s="9" t="s">
+      <c r="E34" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F34" s="7" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="35" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="12" t="s">
+    <row r="35" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B35" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C35" s="12" t="s">
+      <c r="B35" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C35" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="D35" s="12" t="s">
+      <c r="D35" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="E35" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F35" s="12" t="s">
+      <c r="E35" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F35" s="10" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="36" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="9" t="s">
+    <row r="36" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B36" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C36" s="9" t="s">
+      <c r="B36" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C36" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D36" s="9" t="s">
+      <c r="D36" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="E36" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F36" s="9" t="s">
+      <c r="E36" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F36" s="7" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="12" t="s">
+    <row r="37" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B37" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C37" s="12" t="s">
+      <c r="B37" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C37" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="D37" s="12" t="s">
+      <c r="D37" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="E37" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F37" s="12" t="s">
+      <c r="E37" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F37" s="10" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="38" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="9" t="s">
+    <row r="38" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B38" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C38" s="9" t="s">
+      <c r="B38" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C38" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="D38" s="9" t="s">
+      <c r="D38" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="E38" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F38" s="9" t="s">
+      <c r="E38" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F38" s="7" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="12" t="s">
+    <row r="39" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B39" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C39" s="12" t="s">
+      <c r="B39" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C39" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="D39" s="12" t="s">
+      <c r="D39" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="E39" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F39" s="12" t="s">
+      <c r="E39" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F39" s="10" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="40" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="9" t="s">
+    <row r="40" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B40" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C40" s="9" t="s">
+      <c r="B40" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C40" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="D40" s="9" t="s">
+      <c r="D40" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="E40" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F40" s="9" t="s">
+      <c r="E40" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F40" s="7" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="41" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="12" t="s">
+    <row r="41" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B41" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C41" s="12" t="s">
+      <c r="B41" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C41" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="D41" s="12" t="s">
+      <c r="D41" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="E41" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F41" s="12" t="s">
+      <c r="E41" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F41" s="10" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="42" ht="18" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="9" t="s">
+    <row r="42" spans="1:6" s="6" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B42" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C42" s="9" t="s">
+      <c r="B42" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C42" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="D42" s="9" t="s">
+      <c r="D42" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="E42" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="F42" s="9" t="s">
+      <c r="E42" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F42" s="7" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="43" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="12" t="s">
+    <row r="43" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B43" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C43" s="12" t="s">
+      <c r="B43" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C43" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="D43" s="12" t="s">
+      <c r="D43" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="E43" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F43" s="12" t="s">
+      <c r="E43" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F43" s="10" t="s">
         <v>87</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F22"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -1975,448 +1989,448 @@
     <col min="6" max="6" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:6" s="12" customFormat="1" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="13" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+    <row r="2" spans="1:6" s="14" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="D2" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="E2" s="17" t="s">
+      <c r="D2" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="15" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+    <row r="3" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="D3" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E3" s="12" t="s">
+      <c r="D3" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="10" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
+    <row r="4" spans="1:6" s="14" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="D4" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="E4" s="17" t="s">
+      <c r="D4" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="F4" s="17" t="s">
+      <c r="F4" s="15" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+    <row r="5" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="D5" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" s="12" t="s">
+      <c r="D5" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="F5" s="10" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
+    <row r="6" spans="1:6" s="14" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="D6" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="E6" s="17" t="s">
+      <c r="D6" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="F6" s="17" t="s">
+      <c r="F6" s="15" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="7" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+    <row r="7" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="D7" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E7" s="12" t="s">
+      <c r="D7" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="10" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="17" t="s">
+    <row r="8" spans="1:6" s="14" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="D8" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="E8" s="17" t="s">
+      <c r="D8" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="F8" s="17" t="s">
+      <c r="F8" s="15" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
+    <row r="9" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="D9" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E9" s="12" t="s">
+      <c r="D9" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="F9" s="12" t="s">
+      <c r="F9" s="10" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="17" t="s">
+    <row r="10" spans="1:6" s="14" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="D10" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="E10" s="17" t="s">
+      <c r="D10" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E10" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="F10" s="17" t="s">
+      <c r="F10" s="15" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
+    <row r="11" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="D11" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E11" s="12" t="s">
+      <c r="D11" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="F11" s="12" t="s">
+      <c r="F11" s="10" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="17" t="s">
+    <row r="12" spans="1:6" s="14" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="15" t="s">
         <v>132</v>
       </c>
-      <c r="D12" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="E12" s="17" t="s">
+      <c r="D12" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E12" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="F12" s="17" t="s">
+      <c r="F12" s="15" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="12" t="s">
+    <row r="13" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="D13" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E13" s="12" t="s">
+      <c r="D13" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F13" s="12" t="s">
+      <c r="F13" s="10" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
+    <row r="14" spans="1:6" s="14" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="C14" s="17" t="s">
+      <c r="C14" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="D14" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="E14" s="17" t="s">
+      <c r="D14" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="F14" s="17" t="s">
+      <c r="F14" s="15" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
+    <row r="15" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C15" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="D15" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E15" s="12" t="s">
+      <c r="D15" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="E15" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="F15" s="12" t="s">
+      <c r="F15" s="10" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17" t="s">
+    <row r="16" spans="1:6" s="14" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="15" t="s">
         <v>138</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="C16" s="17" t="s">
+      <c r="C16" s="15" t="s">
         <v>142</v>
       </c>
-      <c r="D16" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="E16" s="17" t="s">
+      <c r="D16" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E16" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="F16" s="17" t="s">
+      <c r="F16" s="15" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
+    <row r="17" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C17" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="D17" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E17" s="12" t="s">
+      <c r="D17" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="E17" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="F17" s="12" t="s">
+      <c r="F17" s="10" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="18" ht="18" customHeight="1" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="17" t="s">
+    <row r="18" spans="1:6" s="14" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="15" t="s">
         <v>138</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="C18" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="D18" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="E18" s="17" t="s">
+      <c r="D18" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="F18" s="17" t="s">
+      <c r="F18" s="15" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
+    <row r="19" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="B19" s="12" t="s">
+      <c r="B19" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="C19" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="D19" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E19" s="12" t="s">
+      <c r="D19" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="E19" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="F19" s="12" t="s">
+      <c r="F19" s="10" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="20" ht="18" customHeight="1" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="17" t="s">
+    <row r="20" spans="1:6" s="14" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="15" t="s">
         <v>152</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="D20" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="E20" s="17" t="s">
+      <c r="D20" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E20" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="F20" s="17" t="s">
+      <c r="F20" s="15" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="21" ht="18" customHeight="1" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="12" t="s">
+    <row r="21" spans="1:6" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="10" t="s">
         <v>151</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="B21" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="C21" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="D21" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="E21" s="12" t="s">
+      <c r="D21" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="E21" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="F21" s="12" t="s">
+      <c r="F21" s="10" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="22" ht="18" customHeight="1" spans="1:6" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="17" t="s">
+    <row r="22" spans="1:6" s="14" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="15" t="s">
         <v>152</v>
       </c>
-      <c r="C22" s="17" t="s">
+      <c r="C22" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="D22" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="E22" s="17" t="s">
+      <c r="D22" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="E22" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="F22" s="17" t="s">
+      <c r="F22" s="15" t="s">
         <v>110</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>